<commit_message>
did my arbeitsjournal thingy
</commit_message>
<xml_diff>
--- a/organisation/Arbeitsjournal_m306.xlsx
+++ b/organisation/Arbeitsjournal_m306.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\neo.dijkstra\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alex\source\repos\M306-Projektarbeit\organisation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C13D4941-F5FA-4482-9976-A8EF055AE6D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F972AF4-44EF-4ACF-A44E-94FAF4B540BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{FD90AA82-B1B6-476E-8080-72CCFDD3408C}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="27634" windowHeight="14914" xr2:uid="{FD90AA82-B1B6-476E-8080-72CCFDD3408C}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="86">
   <si>
     <t>Datum</t>
   </si>
@@ -273,6 +273,24 @@
   </si>
   <si>
     <t>Alles ok, ich kann aber schon vorhersehen dass es eventuell Probleme geben wird mit Api parser/satellite orbit renderer und das 3d frontend</t>
+  </si>
+  <si>
+    <t>Verbessern doku</t>
+  </si>
+  <si>
+    <t>Dokumentation automatisch kompiliert</t>
+  </si>
+  <si>
+    <t>Dokumentation kompilieren dauerte ewig</t>
+  </si>
+  <si>
+    <t>Word styles</t>
+  </si>
+  <si>
+    <t>Göggle</t>
+  </si>
+  <si>
+    <t>AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</t>
   </si>
 </sst>
 </file>
@@ -357,7 +375,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -370,14 +388,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0" customBuiltin="1"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -393,7 +406,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -710,14 +723,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E02F4629-0B56-4CEA-A5D3-42C219E50C42}">
   <dimension ref="A1:N44"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="10.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="25.54296875" customWidth="1"/>
-    <col min="2" max="8" width="21.81640625" customWidth="1"/>
-    <col min="9" max="9" width="10.90625" customWidth="1"/>
+    <col min="1" max="1" width="25.53515625" customWidth="1"/>
+    <col min="2" max="8" width="21.84375" customWidth="1"/>
+    <col min="9" max="9" width="10.921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -733,34 +746,28 @@
       <c r="E1" s="2">
         <v>46174</v>
       </c>
-      <c r="F1" s="7">
+      <c r="F1" s="2">
         <v>46181</v>
       </c>
-      <c r="G1" s="7">
+      <c r="G1" s="2">
         <v>46188</v>
       </c>
-      <c r="H1" s="7">
+      <c r="H1" s="2">
         <v>46195</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A2" s="5"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C3" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -773,11 +780,8 @@
       <c r="E4" t="s">
         <v>73</v>
       </c>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -790,11 +794,8 @@
       <c r="E5" t="s">
         <v>74</v>
       </c>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
@@ -807,11 +808,8 @@
       <c r="E6" t="s">
         <v>75</v>
       </c>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
@@ -824,11 +822,8 @@
       <c r="E7" t="s">
         <v>76</v>
       </c>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
@@ -841,9 +836,8 @@
       <c r="E8" t="s">
         <v>77</v>
       </c>
-      <c r="F8" s="6"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
       <c r="K8" s="4"/>
@@ -851,7 +845,7 @@
       <c r="M8" s="4"/>
       <c r="N8" s="4"/>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A9" s="3" t="s">
         <v>7</v>
       </c>
@@ -864,11 +858,8 @@
       <c r="E9" t="s">
         <v>78</v>
       </c>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A10" s="3" t="s">
         <v>8</v>
       </c>
@@ -881,11 +872,8 @@
       <c r="E10" t="s">
         <v>42</v>
       </c>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
@@ -898,11 +886,8 @@
       <c r="E11" t="s">
         <v>79</v>
       </c>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A12" s="5" t="s">
         <v>0</v>
       </c>
@@ -918,34 +903,28 @@
       <c r="E12" s="2">
         <v>46174</v>
       </c>
-      <c r="F12" s="7">
+      <c r="F12" s="2">
         <v>46181</v>
       </c>
-      <c r="G12" s="7">
+      <c r="G12" s="2">
         <v>46188</v>
       </c>
-      <c r="H12" s="7">
+      <c r="H12" s="2">
         <v>46195</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A13" s="5"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A14" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C14" t="s">
         <v>11</v>
       </c>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A15" s="3" t="s">
         <v>2</v>
       </c>
@@ -958,11 +937,8 @@
       <c r="E15" t="s">
         <v>55</v>
       </c>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A16" s="3" t="s">
         <v>3</v>
       </c>
@@ -975,11 +951,8 @@
       <c r="E16" t="s">
         <v>71</v>
       </c>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A17" s="3" t="s">
         <v>4</v>
       </c>
@@ -992,11 +965,8 @@
       <c r="E17" t="s">
         <v>17</v>
       </c>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
-      <c r="H17" s="6"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A18" s="3" t="s">
         <v>5</v>
       </c>
@@ -1009,11 +979,8 @@
       <c r="E18" t="s">
         <v>69</v>
       </c>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="6"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A19" s="3" t="s">
         <v>6</v>
       </c>
@@ -1026,11 +993,10 @@
       <c r="E19" t="s">
         <v>61</v>
       </c>
-      <c r="F19" s="6"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="8"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A20" s="3" t="s">
         <v>7</v>
       </c>
@@ -1043,11 +1009,8 @@
       <c r="E20" t="s">
         <v>17</v>
       </c>
-      <c r="F20" s="6"/>
-      <c r="G20" s="6"/>
-      <c r="H20" s="6"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A21" s="3" t="s">
         <v>8</v>
       </c>
@@ -1060,11 +1023,8 @@
       <c r="E21" t="s">
         <v>70</v>
       </c>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
-      <c r="H21" s="6"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A22" s="3" t="s">
         <v>9</v>
       </c>
@@ -1077,11 +1037,8 @@
       <c r="E22" t="s">
         <v>72</v>
       </c>
-      <c r="F22" s="6"/>
-      <c r="G22" s="6"/>
-      <c r="H22" s="6"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A23" s="5" t="s">
         <v>0</v>
       </c>
@@ -1094,41 +1051,34 @@
       <c r="D23" s="2">
         <v>46160</v>
       </c>
-      <c r="E23" s="7">
+      <c r="E23" s="2">
         <v>46174</v>
       </c>
-      <c r="F23" s="7">
+      <c r="F23" s="2">
         <v>46181</v>
       </c>
-      <c r="G23" s="7">
+      <c r="G23" s="2">
         <v>46188</v>
       </c>
-      <c r="H23" s="7">
+      <c r="H23" s="2">
         <v>46195</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A24" s="5"/>
-      <c r="E24" s="6"/>
-      <c r="F24" s="6"/>
-      <c r="G24" s="6"/>
-      <c r="H24" s="6"/>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A25" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C25" t="s">
         <v>12</v>
       </c>
-      <c r="E25" s="6" t="s">
+      <c r="E25" t="s">
         <v>56</v>
       </c>
-      <c r="F25" s="6"/>
-      <c r="G25" s="6"/>
-      <c r="H25" s="6"/>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A26" s="3" t="s">
         <v>2</v>
       </c>
@@ -1138,14 +1088,11 @@
       <c r="D26" t="s">
         <v>50</v>
       </c>
-      <c r="E26" s="6" t="s">
+      <c r="E26" t="s">
         <v>57</v>
       </c>
-      <c r="F26" s="6"/>
-      <c r="G26" s="6"/>
-      <c r="H26" s="6"/>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A27" s="3" t="s">
         <v>3</v>
       </c>
@@ -1155,14 +1102,11 @@
       <c r="D27" t="s">
         <v>51</v>
       </c>
-      <c r="E27" s="6" t="s">
+      <c r="E27" t="s">
         <v>58</v>
       </c>
-      <c r="F27" s="6"/>
-      <c r="G27" s="6"/>
-      <c r="H27" s="6"/>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A28" s="3" t="s">
         <v>4</v>
       </c>
@@ -1172,14 +1116,11 @@
       <c r="D28" t="s">
         <v>52</v>
       </c>
-      <c r="E28" s="6" t="s">
+      <c r="E28" t="s">
         <v>59</v>
       </c>
-      <c r="F28" s="6"/>
-      <c r="G28" s="6"/>
-      <c r="H28" s="6"/>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A29" s="3" t="s">
         <v>5</v>
       </c>
@@ -1189,14 +1130,11 @@
       <c r="D29" t="s">
         <v>53</v>
       </c>
-      <c r="E29" s="6" t="s">
+      <c r="E29" t="s">
         <v>60</v>
       </c>
-      <c r="F29" s="6"/>
-      <c r="G29" s="6"/>
-      <c r="H29" s="6"/>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A30" s="3" t="s">
         <v>6</v>
       </c>
@@ -1206,14 +1144,13 @@
       <c r="D30" t="s">
         <v>42</v>
       </c>
-      <c r="E30" s="6" t="s">
+      <c r="E30" t="s">
         <v>61</v>
       </c>
-      <c r="F30" s="6"/>
-      <c r="G30" s="8"/>
-      <c r="H30" s="8"/>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="G30" s="4"/>
+      <c r="H30" s="4"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A31" s="3" t="s">
         <v>7</v>
       </c>
@@ -1223,14 +1160,11 @@
       <c r="D31" t="s">
         <v>42</v>
       </c>
-      <c r="E31" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="F31" s="6"/>
-      <c r="G31" s="6"/>
-      <c r="H31" s="6"/>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E31" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A32" s="3" t="s">
         <v>8</v>
       </c>
@@ -1240,14 +1174,11 @@
       <c r="D32" t="s">
         <v>42</v>
       </c>
-      <c r="E32" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="F32" s="6"/>
-      <c r="G32" s="6"/>
-      <c r="H32" s="6"/>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E32" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A33" s="3" t="s">
         <v>9</v>
       </c>
@@ -1257,14 +1188,11 @@
       <c r="D33" t="s">
         <v>54</v>
       </c>
-      <c r="E33" s="6" t="s">
+      <c r="E33" t="s">
         <v>62</v>
       </c>
-      <c r="F33" s="6"/>
-      <c r="G33" s="6"/>
-      <c r="H33" s="6"/>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A34" s="5" t="s">
         <v>0</v>
       </c>
@@ -1277,35 +1205,37 @@
       <c r="D34" s="2">
         <v>46160</v>
       </c>
-      <c r="E34" s="7">
+      <c r="E34" s="2">
         <v>46174</v>
       </c>
-      <c r="F34" s="7">
+      <c r="F34" s="2">
         <v>46181</v>
       </c>
-      <c r="G34" s="7">
+      <c r="G34" s="2">
         <v>46188</v>
       </c>
-      <c r="H34" s="7">
+      <c r="H34" s="2">
         <v>46195</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A35" s="5"/>
-      <c r="E35" s="6"/>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A36" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C36" t="s">
         <v>13</v>
       </c>
-      <c r="E36" s="6" t="s">
+      <c r="E36" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="F36" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A37" s="3" t="s">
         <v>2</v>
       </c>
@@ -1315,11 +1245,14 @@
       <c r="D37" t="s">
         <v>44</v>
       </c>
-      <c r="E37" s="6" t="s">
+      <c r="E37" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="F37" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A38" s="3" t="s">
         <v>3</v>
       </c>
@@ -1329,22 +1262,28 @@
       <c r="D38" t="s">
         <v>45</v>
       </c>
-      <c r="E38" s="6" t="s">
+      <c r="E38" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="F38" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A39" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C39" t="s">
         <v>17</v>
       </c>
-      <c r="E39" s="6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E39" t="s">
+        <v>17</v>
+      </c>
+      <c r="F39" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A40" s="3" t="s">
         <v>5</v>
       </c>
@@ -1354,11 +1293,14 @@
       <c r="D40" t="s">
         <v>46</v>
       </c>
-      <c r="E40" s="6" t="s">
+      <c r="E40" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="F40" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A41" s="3" t="s">
         <v>6</v>
       </c>
@@ -1368,12 +1310,15 @@
       <c r="D41" t="s">
         <v>42</v>
       </c>
-      <c r="E41" s="6" t="s">
+      <c r="E41" t="s">
         <v>67</v>
       </c>
+      <c r="F41" t="s">
+        <v>84</v>
+      </c>
       <c r="H41" s="4"/>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A42" s="3" t="s">
         <v>7</v>
       </c>
@@ -1383,11 +1328,14 @@
       <c r="D42" t="s">
         <v>42</v>
       </c>
-      <c r="E42" s="6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E42" t="s">
+        <v>17</v>
+      </c>
+      <c r="F42" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A43" s="3" t="s">
         <v>8</v>
       </c>
@@ -1397,11 +1345,14 @@
       <c r="D43" t="s">
         <v>42</v>
       </c>
-      <c r="E43" s="6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E43" t="s">
+        <v>17</v>
+      </c>
+      <c r="F43" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A44" s="3" t="s">
         <v>9</v>
       </c>
@@ -1411,8 +1362,11 @@
       <c r="D44" t="s">
         <v>48</v>
       </c>
-      <c r="E44" s="6" t="s">
+      <c r="E44" t="s">
         <v>68</v>
+      </c>
+      <c r="F44" t="s">
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -1428,20 +1382,20 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="c7b2f2ff-66ba-4f36-b635-223a8833b290" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="c7b2f2ff-66ba-4f36-b635-223a8833b290" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1678,6 +1632,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{64E447DC-C281-49C6-9351-47DCD570C246}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3F0D940-730F-41F1-8757-0FBD047F37CA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="c7b2f2ff-66ba-4f36-b635-223a8833b290"/>
@@ -1690,14 +1652,6 @@
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="4271d823-fc57-4cd5-873b-9886274042dd"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{64E447DC-C281-49C6-9351-47DCD570C246}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
updated arbeitsjournal and zeitpan
</commit_message>
<xml_diff>
--- a/organisation/Arbeitsjournal_m306.xlsx
+++ b/organisation/Arbeitsjournal_m306.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vince\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alex\source\repos\M306-Projektarbeit\organisation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB8D5910-BDE1-4E4D-9B81-4A58A76CA1C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96FDC7C9-F1C8-4C49-9730-6834ED516F9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FD90AA82-B1B6-476E-8080-72CCFDD3408C}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="27634" windowHeight="14914" xr2:uid="{FD90AA82-B1B6-476E-8080-72CCFDD3408C}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -33,14 +33,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="121">
   <si>
     <t>Datum</t>
   </si>
   <si>
-    <t>Teammitglied</t>
-  </si>
-  <si>
     <t>Geplannte Tätigkeiten</t>
   </si>
   <si>
@@ -65,18 +62,6 @@
     <t>Reflexion</t>
   </si>
   <si>
-    <t>Neo Dijkstra</t>
-  </si>
-  <si>
-    <t>Laurentiu Berdila</t>
-  </si>
-  <si>
-    <t>Vincent de Vries</t>
-  </si>
-  <si>
-    <t>Alexander Straub</t>
-  </si>
-  <si>
     <t>Arbeitsvorlage erstellen</t>
   </si>
   <si>
@@ -224,9 +209,6 @@
     <t>Heute ging es organisationsmässig viel besser, da wir alle vor ort waren</t>
   </si>
   <si>
-    <t>Alexander</t>
-  </si>
-  <si>
     <t>Hilfe bei programmier arbeit</t>
   </si>
   <si>
@@ -339,6 +321,81 @@
   </si>
   <si>
     <t>Ich bin grundsätzlich gut voran gekommen und bin auch zufrieden mit dem aktuellen Produkt. Leider lagt die Website im Moment stark. Ausserdem hatte ich vergessen am Ende den Code und die aktualisierten Dateien zu pushen.</t>
+  </si>
+  <si>
+    <t>Neo</t>
+  </si>
+  <si>
+    <t>Laurentiu</t>
+  </si>
+  <si>
+    <t>Alex</t>
+  </si>
+  <si>
+    <t>Arbeit an Dokumentation</t>
+  </si>
+  <si>
+    <t>Compiler .md -&gt; .docx</t>
+  </si>
+  <si>
+    <t>Compiler brauchte lange</t>
+  </si>
+  <si>
+    <t>Zeitstress (wir sind hinter zeitplan)</t>
+  </si>
+  <si>
+    <t>Google Gemini</t>
+  </si>
+  <si>
+    <t>Compiler für .md schreiben</t>
+  </si>
+  <si>
+    <t>Heute war es gegen anfang recht langweilig jedoch hatte ich sehr viel spass mit dem Compiler zu word</t>
+  </si>
+  <si>
+    <t>Fertigmachen App</t>
+  </si>
+  <si>
+    <t>Code zusammengetan</t>
+  </si>
+  <si>
+    <t>Heute arbeiten, da hinter zeitplan</t>
+  </si>
+  <si>
+    <t>Git</t>
+  </si>
+  <si>
+    <t>Alles funktionierte grundsätzlich und wir wurden einigermassen fertig, ist aber schade dass wir heute noch code fertig machen mussten</t>
+  </si>
+  <si>
+    <t>Code fertig</t>
+  </si>
+  <si>
+    <t>Code fertigmachen</t>
+  </si>
+  <si>
+    <t>Projekt läuft</t>
+  </si>
+  <si>
+    <t>Zeit schlecht eingeteilt</t>
+  </si>
+  <si>
+    <t>immernoch IP-bans</t>
+  </si>
+  <si>
+    <t>Ich konnte heute den Code fertigmachen und dann auch noch bei der dokumentation fertigarbeiten. Wir hatten ein leichtes chaos mit git aber es funktionierte eigentlich ok</t>
+  </si>
+  <si>
+    <t>Dokumentation fertig</t>
+  </si>
+  <si>
+    <t>Zeitstress</t>
+  </si>
+  <si>
+    <t>Google Gemini, Claude, r/excel</t>
+  </si>
+  <si>
+    <t>Heute musste ich nochmals unter ein wenig zeitdruck die Dokumentation irgendwie fertigbekommen, was recht stressig war</t>
   </si>
 </sst>
 </file>
@@ -434,7 +491,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -770,15 +827,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E02F4629-0B56-4CEA-A5D3-42C219E50C42}">
-  <dimension ref="A1:N44"/>
-  <sheetFormatPr defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:M40"/>
+  <sheetFormatPr defaultColWidth="10.69140625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="25.5703125" customWidth="1"/>
-    <col min="2" max="8" width="21.85546875" customWidth="1"/>
-    <col min="9" max="9" width="10.85546875" customWidth="1"/>
+    <col min="1" max="1" width="25.53515625" customWidth="1"/>
+    <col min="2" max="7" width="21.84375" customWidth="1"/>
+    <col min="8" max="8" width="10.84375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -800,690 +857,737 @@
       <c r="G1" s="2">
         <v>46188</v>
       </c>
-      <c r="H1" s="2">
-        <v>46195</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="5"/>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="A2" s="5" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" t="s">
+        <v>67</v>
+      </c>
+      <c r="F3" t="s">
+        <v>81</v>
+      </c>
+      <c r="G3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D4" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E4" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F4" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+      <c r="G4" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E5" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F5" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+        <v>83</v>
+      </c>
+      <c r="G5" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D6" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="E6" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F6" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+        <v>84</v>
+      </c>
+      <c r="G6" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D7" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E7" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="F7" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+        <v>85</v>
+      </c>
+      <c r="G7" t="s">
+        <v>85</v>
+      </c>
+      <c r="H7" s="4"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="4"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="4"/>
+      <c r="M7" s="4"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D8" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="E8" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="F8" t="s">
-        <v>91</v>
-      </c>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
-      <c r="M8" s="4"/>
-      <c r="N8" s="4"/>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+        <v>86</v>
+      </c>
+      <c r="G8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A9" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C9" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="D9" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E9" t="s">
-        <v>78</v>
+        <v>37</v>
       </c>
       <c r="F9" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="G9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A10" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" t="s">
+        <v>42</v>
+      </c>
+      <c r="E10" t="s">
+        <v>73</v>
+      </c>
+      <c r="F10" t="s">
+        <v>87</v>
+      </c>
+      <c r="G10" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="A11" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B11" s="1">
+        <v>46146</v>
+      </c>
+      <c r="C11" s="2">
+        <v>46153</v>
+      </c>
+      <c r="D11" s="2">
+        <v>46160</v>
+      </c>
+      <c r="E11" s="2">
+        <v>46174</v>
+      </c>
+      <c r="F11" s="2">
+        <v>46181</v>
+      </c>
+      <c r="G11" s="2">
+        <v>46188</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="A12" s="5" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="A13" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" t="s">
+        <v>44</v>
+      </c>
+      <c r="E13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F13" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="A14" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C14" t="s">
+        <v>21</v>
+      </c>
+      <c r="D14" t="s">
+        <v>32</v>
+      </c>
+      <c r="E14" t="s">
+        <v>65</v>
+      </c>
+      <c r="F14" t="s">
+        <v>75</v>
+      </c>
+      <c r="G14" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="A15" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C15" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" t="s">
+        <v>76</v>
+      </c>
+      <c r="G15" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="A16" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" t="s">
+        <v>63</v>
+      </c>
+      <c r="F16" t="s">
+        <v>77</v>
+      </c>
+      <c r="G16" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A17" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C17" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17" t="s">
+        <v>56</v>
+      </c>
+      <c r="F17" t="s">
+        <v>79</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A18" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" t="s">
+        <v>12</v>
+      </c>
+      <c r="F18" t="s">
+        <v>78</v>
+      </c>
+      <c r="G18" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A19" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D19" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" t="s">
+        <v>64</v>
+      </c>
+      <c r="G19" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A20" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" t="s">
+        <v>25</v>
+      </c>
+      <c r="D20" t="s">
+        <v>33</v>
+      </c>
+      <c r="E20" t="s">
+        <v>66</v>
+      </c>
+      <c r="F20" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A21" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B21" s="1">
+        <v>46146</v>
+      </c>
+      <c r="C21" s="2">
+        <v>46153</v>
+      </c>
+      <c r="D21" s="2">
+        <v>46160</v>
+      </c>
+      <c r="E21" s="2">
+        <v>46174</v>
+      </c>
+      <c r="F21" s="2">
+        <v>46181</v>
+      </c>
+      <c r="G21" s="2">
+        <v>46188</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A22" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A23" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>31</v>
+      </c>
+      <c r="D23" t="s">
+        <v>45</v>
+      </c>
+      <c r="E23" t="s">
+        <v>52</v>
+      </c>
+      <c r="F23" t="s">
+        <v>89</v>
+      </c>
+      <c r="G23" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A24" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C24" t="s">
         <v>17</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D24" t="s">
+        <v>46</v>
+      </c>
+      <c r="E24" t="s">
+        <v>53</v>
+      </c>
+      <c r="F24" t="s">
+        <v>88</v>
+      </c>
+      <c r="G24" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A25" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C25" t="s">
+        <v>18</v>
+      </c>
+      <c r="D25" t="s">
+        <v>47</v>
+      </c>
+      <c r="E25" t="s">
+        <v>54</v>
+      </c>
+      <c r="F25" t="s">
+        <v>93</v>
+      </c>
+      <c r="G25" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A26" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C26" t="s">
+        <v>16</v>
+      </c>
+      <c r="D26" t="s">
+        <v>48</v>
+      </c>
+      <c r="E26" t="s">
+        <v>55</v>
+      </c>
+      <c r="F26" t="s">
+        <v>94</v>
+      </c>
+      <c r="G26" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A27" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C27" t="s">
+        <v>12</v>
+      </c>
+      <c r="D27" t="s">
+        <v>37</v>
+      </c>
+      <c r="E27" t="s">
+        <v>56</v>
+      </c>
+      <c r="F27" t="s">
+        <v>90</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A28" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C28" t="s">
+        <v>12</v>
+      </c>
+      <c r="D28" t="s">
+        <v>37</v>
+      </c>
+      <c r="E28" t="s">
+        <v>12</v>
+      </c>
+      <c r="F28" t="s">
+        <v>91</v>
+      </c>
+      <c r="G28" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A29" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C29" t="s">
+        <v>19</v>
+      </c>
+      <c r="D29" t="s">
+        <v>37</v>
+      </c>
+      <c r="E29" t="s">
+        <v>12</v>
+      </c>
+      <c r="F29" t="s">
+        <v>92</v>
+      </c>
+      <c r="G29" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A30" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C30" t="s">
+        <v>24</v>
+      </c>
+      <c r="D30" t="s">
+        <v>49</v>
+      </c>
+      <c r="E30" t="s">
+        <v>57</v>
+      </c>
+      <c r="F30" t="s">
+        <v>95</v>
+      </c>
+      <c r="G30" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A31" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B31" s="1">
+        <v>46146</v>
+      </c>
+      <c r="C31" s="2">
+        <v>46153</v>
+      </c>
+      <c r="D31" s="2">
+        <v>46160</v>
+      </c>
+      <c r="E31" s="2">
+        <v>46174</v>
+      </c>
+      <c r="F31" s="2">
+        <v>46181</v>
+      </c>
+      <c r="G31" s="2">
+        <v>46188</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A32" s="5" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A33" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C33" t="s">
+        <v>22</v>
+      </c>
+      <c r="D33" t="s">
+        <v>39</v>
+      </c>
+      <c r="E33" t="s">
+        <v>58</v>
+      </c>
+      <c r="F33" t="s">
+        <v>99</v>
+      </c>
+      <c r="G33" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A34" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>23</v>
+      </c>
+      <c r="D34" t="s">
+        <v>40</v>
+      </c>
+      <c r="E34" t="s">
+        <v>59</v>
+      </c>
+      <c r="F34" t="s">
+        <v>100</v>
+      </c>
+      <c r="G34" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A35" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C35" t="s">
+        <v>12</v>
+      </c>
+      <c r="E35" t="s">
+        <v>12</v>
+      </c>
+      <c r="F35" t="s">
+        <v>101</v>
+      </c>
+      <c r="G35" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A36" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C36" t="s">
+        <v>27</v>
+      </c>
+      <c r="D36" t="s">
+        <v>41</v>
+      </c>
+      <c r="E36" t="s">
+        <v>60</v>
+      </c>
+      <c r="F36" t="s">
+        <v>102</v>
+      </c>
+      <c r="G36" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A37" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C37" t="s">
+        <v>12</v>
+      </c>
+      <c r="D37" t="s">
+        <v>37</v>
+      </c>
+      <c r="E37" t="s">
+        <v>61</v>
+      </c>
+      <c r="F37" t="s">
+        <v>103</v>
+      </c>
+      <c r="G37" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A38" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C38" t="s">
+        <v>12</v>
+      </c>
+      <c r="D38" t="s">
+        <v>37</v>
+      </c>
+      <c r="E38" t="s">
+        <v>12</v>
+      </c>
+      <c r="F38" t="s">
+        <v>12</v>
+      </c>
+      <c r="G38" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A39" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C39" t="s">
+        <v>12</v>
+      </c>
+      <c r="D39" t="s">
+        <v>37</v>
+      </c>
+      <c r="E39" t="s">
+        <v>12</v>
+      </c>
+      <c r="F39" t="s">
+        <v>104</v>
+      </c>
+      <c r="G39" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A40" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C40" t="s">
+        <v>28</v>
+      </c>
+      <c r="D40" t="s">
         <v>43</v>
       </c>
-      <c r="E10" t="s">
-        <v>42</v>
-      </c>
-      <c r="F10" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C11" t="s">
-        <v>20</v>
-      </c>
-      <c r="D11" t="s">
-        <v>47</v>
-      </c>
-      <c r="E11" t="s">
-        <v>79</v>
-      </c>
-      <c r="F11" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B12" s="1">
-        <v>46146</v>
-      </c>
-      <c r="C12" s="2">
-        <v>46153</v>
-      </c>
-      <c r="D12" s="2">
-        <v>46160</v>
-      </c>
-      <c r="E12" s="2">
-        <v>46174</v>
-      </c>
-      <c r="F12" s="2">
-        <v>46181</v>
-      </c>
-      <c r="G12" s="2">
-        <v>46188</v>
-      </c>
-      <c r="H12" s="2">
-        <v>46195</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="5"/>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C14" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C15" t="s">
-        <v>25</v>
-      </c>
-      <c r="D15" t="s">
-        <v>49</v>
-      </c>
-      <c r="E15" t="s">
-        <v>55</v>
-      </c>
-      <c r="F15" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C16" t="s">
-        <v>26</v>
-      </c>
-      <c r="D16" t="s">
-        <v>37</v>
-      </c>
-      <c r="E16" t="s">
-        <v>71</v>
-      </c>
-      <c r="F16" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C17" t="s">
-        <v>17</v>
-      </c>
-      <c r="D17" t="s">
-        <v>17</v>
-      </c>
-      <c r="E17" t="s">
-        <v>17</v>
-      </c>
-      <c r="F17" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C18" t="s">
-        <v>17</v>
-      </c>
-      <c r="D18" t="s">
-        <v>17</v>
-      </c>
-      <c r="E18" t="s">
-        <v>69</v>
-      </c>
-      <c r="F18" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C19" t="s">
-        <v>17</v>
-      </c>
-      <c r="D19" t="s">
-        <v>39</v>
-      </c>
-      <c r="E19" t="s">
-        <v>61</v>
-      </c>
-      <c r="F19" t="s">
-        <v>85</v>
-      </c>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C20" t="s">
-        <v>17</v>
-      </c>
-      <c r="D20" t="s">
-        <v>17</v>
-      </c>
-      <c r="E20" t="s">
-        <v>17</v>
-      </c>
-      <c r="F20" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C21" t="s">
-        <v>31</v>
-      </c>
-      <c r="D21" t="s">
-        <v>17</v>
-      </c>
-      <c r="E21" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C22" t="s">
-        <v>30</v>
-      </c>
-      <c r="D22" t="s">
-        <v>38</v>
-      </c>
-      <c r="E22" t="s">
-        <v>72</v>
-      </c>
-      <c r="F22" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B23" s="1">
-        <v>46146</v>
-      </c>
-      <c r="C23" s="2">
-        <v>46153</v>
-      </c>
-      <c r="D23" s="2">
-        <v>46160</v>
-      </c>
-      <c r="E23" s="2">
-        <v>46174</v>
-      </c>
-      <c r="F23" s="2">
-        <v>46181</v>
-      </c>
-      <c r="G23" s="2">
-        <v>46188</v>
-      </c>
-      <c r="H23" s="2">
-        <v>46195</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="5"/>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C25" t="s">
-        <v>12</v>
-      </c>
-      <c r="E25" t="s">
-        <v>56</v>
-      </c>
-      <c r="F25" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C26" t="s">
-        <v>36</v>
-      </c>
-      <c r="D26" t="s">
-        <v>50</v>
-      </c>
-      <c r="E26" t="s">
-        <v>57</v>
-      </c>
-      <c r="F26" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C27" t="s">
-        <v>22</v>
-      </c>
-      <c r="D27" t="s">
-        <v>51</v>
-      </c>
-      <c r="E27" t="s">
-        <v>58</v>
-      </c>
-      <c r="F27" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C28" t="s">
-        <v>23</v>
-      </c>
-      <c r="D28" t="s">
-        <v>52</v>
-      </c>
-      <c r="E28" t="s">
-        <v>59</v>
-      </c>
-      <c r="F28" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C29" t="s">
-        <v>21</v>
-      </c>
-      <c r="D29" t="s">
-        <v>53</v>
-      </c>
-      <c r="E29" t="s">
-        <v>60</v>
-      </c>
-      <c r="F29" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C30" t="s">
-        <v>17</v>
-      </c>
-      <c r="D30" t="s">
-        <v>42</v>
-      </c>
-      <c r="E30" t="s">
-        <v>61</v>
-      </c>
-      <c r="F30" t="s">
-        <v>96</v>
-      </c>
-      <c r="G30" s="4"/>
-      <c r="H30" s="4"/>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C31" t="s">
-        <v>17</v>
-      </c>
-      <c r="D31" t="s">
-        <v>42</v>
-      </c>
-      <c r="E31" t="s">
-        <v>17</v>
-      </c>
-      <c r="F31" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C32" t="s">
-        <v>24</v>
-      </c>
-      <c r="D32" t="s">
-        <v>42</v>
-      </c>
-      <c r="E32" t="s">
-        <v>17</v>
-      </c>
-      <c r="F32" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C33" t="s">
-        <v>29</v>
-      </c>
-      <c r="D33" t="s">
-        <v>54</v>
-      </c>
-      <c r="E33" t="s">
+      <c r="E40" t="s">
         <v>62</v>
       </c>
-      <c r="F33" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B34" s="1">
-        <v>46146</v>
-      </c>
-      <c r="C34" s="2">
-        <v>46153</v>
-      </c>
-      <c r="D34" s="2">
-        <v>46160</v>
-      </c>
-      <c r="E34" s="2">
-        <v>46174</v>
-      </c>
-      <c r="F34" s="2">
-        <v>46181</v>
-      </c>
-      <c r="G34" s="2">
-        <v>46188</v>
-      </c>
-      <c r="H34" s="2">
-        <v>46195</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="5"/>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C36" t="s">
-        <v>13</v>
-      </c>
-      <c r="E36" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C37" t="s">
-        <v>27</v>
-      </c>
-      <c r="D37" t="s">
-        <v>44</v>
-      </c>
-      <c r="E37" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C38" t="s">
-        <v>28</v>
-      </c>
-      <c r="D38" t="s">
-        <v>45</v>
-      </c>
-      <c r="E38" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A39" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C39" t="s">
-        <v>17</v>
-      </c>
-      <c r="E39" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A40" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C40" t="s">
-        <v>32</v>
-      </c>
-      <c r="D40" t="s">
-        <v>46</v>
-      </c>
-      <c r="E40" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A41" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C41" t="s">
-        <v>17</v>
-      </c>
-      <c r="D41" t="s">
-        <v>42</v>
-      </c>
-      <c r="E41" t="s">
-        <v>67</v>
-      </c>
-      <c r="H41" s="4"/>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A42" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C42" t="s">
-        <v>17</v>
-      </c>
-      <c r="D42" t="s">
-        <v>42</v>
-      </c>
-      <c r="E42" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A43" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C43" t="s">
-        <v>17</v>
-      </c>
-      <c r="D43" t="s">
-        <v>42</v>
-      </c>
-      <c r="E43" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A44" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C44" t="s">
-        <v>33</v>
-      </c>
-      <c r="D44" t="s">
-        <v>48</v>
-      </c>
-      <c r="E44" t="s">
-        <v>68</v>
+      <c r="F40" t="s">
+        <v>105</v>
+      </c>
+      <c r="G40" t="s">
+        <v>120</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="A34:A35"/>
-  </mergeCells>
   <pageMargins left="0.70000000000000007" right="0.70000000000000007" top="0.78740157500000008" bottom="0.78740157500000008" header="0.30000000000000004" footer="0.30000000000000004"/>
   <pageSetup paperSize="0" fitToWidth="0" fitToHeight="0" orientation="portrait" horizontalDpi="0" verticalDpi="0" copies="0"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100B3CDF11B2DD334468F0D4D4DCCD872D3" ma:contentTypeVersion="15" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="4ec007deb773a0e18af256e90b59dc82">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="c7b2f2ff-66ba-4f36-b635-223a8833b290" xmlns:ns4="4271d823-fc57-4cd5-873b-9886274042dd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b7bd3f88c579eb75c6ccf09e1dc8d76b" ns3:_="" ns4:_="">
     <xsd:import namespace="c7b2f2ff-66ba-4f36-b635-223a8833b290"/>
@@ -1716,6 +1820,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1725,14 +1838,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{64E447DC-C281-49C6-9351-47DCD570C246}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5CDFFB7-3DFA-44DE-8859-FCC9E91B6A68}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1748,6 +1853,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{64E447DC-C281-49C6-9351-47DCD570C246}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>